<commit_message>
Add payment method and delivery time analysis to cleaned sales data
- Analyzed payment methods used across transactions
- Calculated days of delivery using date subtraction
- Built on top of the cleaned/standardized dataset from previous step
</commit_message>
<xml_diff>
--- a/Data Cleaning in Excel Using Power Query/Data Cleaning With Power Query.xlsx
+++ b/Data Cleaning in Excel Using Power Query/Data Cleaning With Power Query.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerwi\OneDrive\Desktop\August\Github Repo\power-query-data-cleaning-automation\Data Cleaning in Excel Using Power Query\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCCD6F5-C448-4629-8AE1-0C77A48E700F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469133D8-166A-4CEE-B3E1-14342F59A73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{FEE65628-DBDE-4F80-BC49-254F637B450D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FEE65628-DBDE-4F80-BC49-254F637B450D}"/>
   </bookViews>
   <sheets>
     <sheet name="Payment Analysis" sheetId="4" r:id="rId1"/>
@@ -425,7 +425,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,17 +458,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -559,7 +569,7 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{F699884A-24BA-4668-A3C2-7CFD816951A9}" uniqueName="1" name="Payment Type" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{2EE425F3-9EC6-45B3-9893-76B9C171F198}" uniqueName="2" name="Average Revenue" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{78B146EC-9D21-4B9F-9361-1D4F9C59AAEF}" uniqueName="3" name="Average Profit Margin" queryTableFieldId="3"/>
+    <tableColumn id="3" xr3:uid="{78B146EC-9D21-4B9F-9361-1D4F9C59AAEF}" uniqueName="3" name="Average Profit Margin" queryTableFieldId="3" dataCellStyle="Percent"/>
     <tableColumn id="4" xr3:uid="{F4D2C25F-63E7-4FD4-97D8-BAC76EA75DC6}" uniqueName="4" name="Count" queryTableFieldId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -964,7 +974,7 @@
       <c r="B2">
         <v>32234.642857142855</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="4">
         <v>0.75923797727757858</v>
       </c>
       <c r="D2">
@@ -978,7 +988,7 @@
       <c r="B3">
         <v>34282.117647058825</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>0.51103369944281229</v>
       </c>
       <c r="D3">

</xml_diff>